<commit_message>
test: update test data for report for emu >3.5.0
</commit_message>
<xml_diff>
--- a/data/test_report/emu.xlsx
+++ b/data/test_report/emu.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="85">
   <si>
     <t>report_date</t>
   </si>
@@ -89,19 +89,19 @@
     <t>/usr/local/bin/docker</t>
   </si>
   <si>
-    <t>dev</t>
-  </si>
-  <si>
-    <t>krona:2024-05-13</t>
-  </si>
-  <si>
-    <t>emu:2025-03-24</t>
+    <t>1.0.0</t>
+  </si>
+  <si>
+    <t>hydragenetics/krona:2025-04-09</t>
+  </si>
+  <si>
+    <t>emu:2025-11-18</t>
   </si>
   <si>
     <t>map-ont</t>
   </si>
   <si>
-    <t>16S</t>
+    <t>emu-prebuilt</t>
   </si>
   <si>
     <t>0.0001</t>
@@ -131,7 +131,7 @@
     <t>0.01</t>
   </si>
   <si>
-    <t>3.4.5</t>
+    <t>3.5.4</t>
   </si>
   <si>
     <t>2.8.1</t>
@@ -140,13 +140,13 @@
     <t>#filtered</t>
   </si>
   <si>
-    <t>#assigned</t>
-  </si>
-  <si>
-    <t>#unassigned</t>
-  </si>
-  <si>
-    <t>prop_assigned</t>
+    <t>#unmapped</t>
+  </si>
+  <si>
+    <t>#mapped_unclassified</t>
+  </si>
+  <si>
+    <t>%assigned</t>
   </si>
   <si>
     <t>barcode01</t>
@@ -185,7 +185,10 @@
     <t>Staphylococcus epidermidis</t>
   </si>
   <si>
-    <t>unassigned</t>
+    <t>unmapped</t>
+  </si>
+  <si>
+    <t>mapped_unclassified</t>
   </si>
   <si>
     <t>total</t>
@@ -200,91 +203,70 @@
     <t>Escherichia coli</t>
   </si>
   <si>
+    <t>Bacillus megaterium</t>
+  </si>
+  <si>
     <t>Leucobacter aridicollis</t>
   </si>
   <si>
-    <t>Bacillus sp. IHB B 7164</t>
-  </si>
-  <si>
-    <t>Bacillus megaterium</t>
-  </si>
-  <si>
-    <t>genus</t>
-  </si>
-  <si>
-    <t>family</t>
-  </si>
-  <si>
-    <t>order</t>
-  </si>
-  <si>
-    <t>class</t>
-  </si>
-  <si>
-    <t>phylum</t>
-  </si>
-  <si>
-    <t>superkingdom</t>
+    <t>Imtechella</t>
   </si>
   <si>
     <t>Staphylococcus</t>
   </si>
   <si>
-    <t xml:space="preserve">Imtechella </t>
-  </si>
-  <si>
     <t>Escherichia</t>
   </si>
   <si>
+    <t>Bacillus</t>
+  </si>
+  <si>
     <t>Leucobacter</t>
   </si>
   <si>
-    <t>Bacillus</t>
+    <t>Flavobacteriaceae</t>
   </si>
   <si>
     <t>Staphylococcaceae</t>
   </si>
   <si>
-    <t>Flavobacteriaceae</t>
-  </si>
-  <si>
     <t>Enterobacteriaceae</t>
   </si>
   <si>
+    <t>Bacillaceae</t>
+  </si>
+  <si>
     <t>Microbacteriaceae</t>
   </si>
   <si>
-    <t>Bacillaceae</t>
+    <t>Flavobacteriales</t>
   </si>
   <si>
     <t>Bacillales</t>
   </si>
   <si>
-    <t>Flavobacteriales</t>
-  </si>
-  <si>
     <t>Enterobacterales</t>
   </si>
   <si>
     <t>Micrococcales</t>
   </si>
   <si>
+    <t>Flavobacteriia</t>
+  </si>
+  <si>
     <t>Bacilli</t>
   </si>
   <si>
-    <t>Flavobacteriia</t>
-  </si>
-  <si>
     <t>Gammaproteobacteria</t>
   </si>
   <si>
     <t>Actinobacteria</t>
   </si>
   <si>
+    <t>Bacteroidota</t>
+  </si>
+  <si>
     <t>Firmicutes</t>
-  </si>
-  <si>
-    <t>Bacteroidota</t>
   </si>
   <si>
     <t>Proteobacteria</t>
@@ -680,7 +662,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2">
-        <v>45758.65994086969</v>
+        <v>45980.46939538528</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -852,7 +834,7 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:F21">
+  <conditionalFormatting sqref="B2:F25">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Imtechella halotolerans">
       <formula>NOT(ISERROR(SEARCH("Imtechella halotolerans",B2)))</formula>
     </cfRule>
@@ -894,16 +876,16 @@
         <v>43</v>
       </c>
       <c r="B2">
-        <v>2700</v>
+        <v>7730</v>
       </c>
       <c r="C2">
-        <v>2700</v>
+        <v>0</v>
       </c>
       <c r="D2">
         <v>0</v>
       </c>
       <c r="E2">
-        <v>1</v>
+        <v>100</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -911,16 +893,16 @@
         <v>44</v>
       </c>
       <c r="B3">
-        <v>2000</v>
+        <v>8620</v>
       </c>
       <c r="C3">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="D3">
         <v>0</v>
       </c>
       <c r="E3">
-        <v>1</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -931,13 +913,13 @@
         <v>1000</v>
       </c>
       <c r="C4">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="D4">
         <v>0</v>
       </c>
       <c r="E4">
-        <v>1</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -945,16 +927,16 @@
         <v>46</v>
       </c>
       <c r="B5">
-        <v>1635</v>
+        <v>1449</v>
       </c>
       <c r="C5">
-        <v>135</v>
+        <v>1304</v>
       </c>
       <c r="D5">
-        <v>1500</v>
+        <v>10</v>
       </c>
       <c r="E5">
-        <v>0.08</v>
+        <v>9.32</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -962,20 +944,20 @@
         <v>47</v>
       </c>
       <c r="B6">
-        <v>110</v>
+        <v>22</v>
       </c>
       <c r="C6">
-        <v>55</v>
+        <v>0</v>
       </c>
       <c r="D6">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E6">
-        <v>0.5</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:F21">
+  <conditionalFormatting sqref="B2:F25">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Imtechella halotolerans">
       <formula>NOT(ISERROR(SEARCH("Imtechella halotolerans",B2)))</formula>
     </cfRule>
@@ -992,7 +974,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.7109375" style="1" customWidth="1"/>
@@ -1030,7 +1012,7 @@
         <v>1</v>
       </c>
       <c r="D2" s="3">
-        <v>2700</v>
+        <v>7730</v>
       </c>
       <c r="E2" s="3">
         <v>1</v>
@@ -1059,353 +1041,433 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:6" s="4" customFormat="1">
-      <c r="A4" s="4" t="s">
+    <row r="4" spans="1:6">
+      <c r="A4" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" t="s">
         <v>56</v>
       </c>
-      <c r="D4" s="4">
-        <v>2700</v>
-      </c>
-      <c r="E4" s="4">
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" s="4" customFormat="1">
+      <c r="A5" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D5" s="4">
+        <v>7730</v>
+      </c>
+      <c r="E5" s="4">
         <v>1</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F5" s="4">
         <v>100</v>
       </c>
     </row>
-    <row r="5" spans="1:6" s="3" customFormat="1">
-      <c r="A5" s="3" t="s">
+    <row r="6" spans="1:6" s="3" customFormat="1">
+      <c r="A6" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B6" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C6" s="3">
+        <v>1</v>
+      </c>
+      <c r="D6" s="3">
+        <v>8620</v>
+      </c>
+      <c r="E6" s="3">
+        <v>1</v>
+      </c>
+      <c r="F6" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B7" t="s">
+        <v>55</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" s="4" customFormat="1">
+      <c r="A9" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="C5" s="3">
+      <c r="D9" s="4">
+        <v>8620</v>
+      </c>
+      <c r="E9" s="4">
         <v>1</v>
       </c>
-      <c r="D5" s="3">
-        <v>2000</v>
-      </c>
-      <c r="E5" s="3">
-        <v>1</v>
-      </c>
-      <c r="F5" s="3">
+      <c r="F9" s="4">
         <v>100</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
-      <c r="A6" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="B6" t="s">
+    <row r="10" spans="1:6" s="3" customFormat="1">
+      <c r="A10" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C10" s="3">
+        <v>95</v>
+      </c>
+      <c r="D10" s="3">
+        <v>950</v>
+      </c>
+      <c r="E10" s="3">
+        <v>0.95</v>
+      </c>
+      <c r="F10" s="3">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" s="3" customFormat="1">
+      <c r="A11" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C11" s="3">
+        <v>5</v>
+      </c>
+      <c r="D11" s="3">
+        <v>50</v>
+      </c>
+      <c r="E11" s="3">
+        <v>0.05</v>
+      </c>
+      <c r="F11" s="3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B12" t="s">
         <v>55</v>
       </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-      <c r="D6">
-        <v>0</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
-      <c r="F6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" s="4" customFormat="1">
-      <c r="A7" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="D7" s="4">
-        <v>2000</v>
-      </c>
-      <c r="E7" s="4">
-        <v>1</v>
-      </c>
-      <c r="F7" s="4">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" s="3" customFormat="1">
-      <c r="A8" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="C8" s="3">
-        <v>0.95</v>
-      </c>
-      <c r="D8" s="3">
-        <v>950</v>
-      </c>
-      <c r="E8" s="3">
-        <v>0.95</v>
-      </c>
-      <c r="F8" s="3">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" s="3" customFormat="1">
-      <c r="A9" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C9" s="3">
-        <v>0.05</v>
-      </c>
-      <c r="D9" s="3">
-        <v>50</v>
-      </c>
-      <c r="E9" s="3">
-        <v>0.05</v>
-      </c>
-      <c r="F9" s="3">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="A10" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="B10" t="s">
-        <v>55</v>
-      </c>
-      <c r="C10">
-        <v>0</v>
-      </c>
-      <c r="D10">
-        <v>0</v>
-      </c>
-      <c r="E10">
-        <v>0</v>
-      </c>
-      <c r="F10">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" s="4" customFormat="1">
-      <c r="A11" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="D11" s="4">
-        <v>1000</v>
-      </c>
-      <c r="E11" s="4">
-        <v>1</v>
-      </c>
-      <c r="F11" s="4">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" s="5" customFormat="1">
-      <c r="A12" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B12" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="C12" s="5">
-        <v>0</v>
-      </c>
-      <c r="D12" s="5">
-        <v>1500</v>
-      </c>
-      <c r="E12" s="5">
-        <v>0.92</v>
-      </c>
-      <c r="F12" s="5">
-        <v>91.73999999999999</v>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="B13" t="s">
+        <v>56</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" s="4" customFormat="1">
+      <c r="A14" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D14" s="4">
+        <v>1000</v>
+      </c>
+      <c r="E14" s="4">
+        <v>1</v>
+      </c>
+      <c r="F14" s="4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" s="5" customFormat="1">
+      <c r="A15" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B13" t="s">
-        <v>59</v>
-      </c>
-      <c r="C13">
+      <c r="B15" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="C15" s="5">
+        <v>0</v>
+      </c>
+      <c r="D15" s="5">
+        <v>1304</v>
+      </c>
+      <c r="E15" s="5">
+        <v>0.9</v>
+      </c>
+      <c r="F15" s="5">
+        <v>89.98999999999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B16" t="s">
+        <v>60</v>
+      </c>
+      <c r="C16">
         <v>0.74</v>
       </c>
-      <c r="D13">
+      <c r="D16">
         <v>100</v>
       </c>
-      <c r="E13">
-        <v>0.06</v>
-      </c>
-      <c r="F13">
-        <v>6.12</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6">
-      <c r="A14" s="1" t="s">
+      <c r="E16">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="F16">
+        <v>6.9</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B17" t="s">
         <v>54</v>
       </c>
-      <c r="C14">
+      <c r="C17">
         <v>0.19</v>
       </c>
-      <c r="D14">
+      <c r="D17">
         <v>25</v>
       </c>
-      <c r="E14">
+      <c r="E17">
         <v>0.02</v>
       </c>
-      <c r="F14">
-        <v>1.53</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6">
-      <c r="A15" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="B15" t="s">
-        <v>58</v>
-      </c>
-      <c r="C15">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="D15">
-        <v>10</v>
-      </c>
-      <c r="E15">
-        <v>0.01</v>
-      </c>
-      <c r="F15">
-        <v>0.61</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" s="4" customFormat="1">
-      <c r="A16" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="D16" s="4">
-        <v>1635</v>
-      </c>
-      <c r="E16" s="4">
-        <v>1</v>
-      </c>
-      <c r="F16" s="4">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" s="3" customFormat="1">
-      <c r="A17" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C17" s="3">
-        <v>0.91</v>
-      </c>
-      <c r="D17" s="3">
-        <v>50</v>
-      </c>
-      <c r="E17" s="3">
-        <v>0.48</v>
-      </c>
-      <c r="F17" s="3">
-        <v>47.62</v>
+      <c r="F17">
+        <v>1.73</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B18" t="s">
+        <v>59</v>
+      </c>
+      <c r="C18">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="D18">
+        <v>10</v>
+      </c>
+      <c r="E18">
+        <v>0.01</v>
+      </c>
+      <c r="F18">
+        <v>0.6899999999999999</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" s="5" customFormat="1">
+      <c r="A19" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C19" s="5">
+        <v>0</v>
+      </c>
+      <c r="D19" s="5">
+        <v>10</v>
+      </c>
+      <c r="E19" s="5">
+        <v>0.01</v>
+      </c>
+      <c r="F19" s="5">
+        <v>0.6899999999999999</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" s="4" customFormat="1">
+      <c r="A20" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D20" s="4">
+        <v>1449</v>
+      </c>
+      <c r="E20" s="4">
+        <v>1</v>
+      </c>
+      <c r="F20" s="4">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6">
+      <c r="A21" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B21" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21">
+        <v>0.59</v>
+      </c>
+      <c r="D21">
+        <v>13</v>
+      </c>
+      <c r="E21">
+        <v>0.59</v>
+      </c>
+      <c r="F21">
+        <v>59.09</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6">
+      <c r="A22" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B22" t="s">
+        <v>62</v>
+      </c>
+      <c r="C22">
+        <v>0.41</v>
+      </c>
+      <c r="D22">
+        <v>9</v>
+      </c>
+      <c r="E22">
+        <v>0.41</v>
+      </c>
+      <c r="F22">
+        <v>40.91</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6">
+      <c r="A23" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B23" t="s">
         <v>55</v>
       </c>
-      <c r="C18">
-        <v>0</v>
-      </c>
-      <c r="D18">
-        <v>50</v>
-      </c>
-      <c r="E18">
-        <v>0.48</v>
-      </c>
-      <c r="F18">
-        <v>47.62</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6">
-      <c r="A19" s="1" t="s">
+      <c r="C23">
+        <v>0</v>
+      </c>
+      <c r="D23">
+        <v>0</v>
+      </c>
+      <c r="E23">
+        <v>0</v>
+      </c>
+      <c r="F23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6">
+      <c r="A24" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B19" t="s">
-        <v>61</v>
-      </c>
-      <c r="C19">
-        <v>0.05</v>
-      </c>
-      <c r="D19">
-        <v>2.77</v>
-      </c>
-      <c r="E19">
-        <v>0.03</v>
-      </c>
-      <c r="F19">
-        <v>2.64</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6">
-      <c r="A20" s="1" t="s">
+      <c r="B24" t="s">
+        <v>56</v>
+      </c>
+      <c r="C24">
+        <v>0</v>
+      </c>
+      <c r="D24">
+        <v>0</v>
+      </c>
+      <c r="E24">
+        <v>0</v>
+      </c>
+      <c r="F24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" s="6" customFormat="1">
+      <c r="A25" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="B20" t="s">
-        <v>62</v>
-      </c>
-      <c r="C20">
-        <v>0.04</v>
-      </c>
-      <c r="D20">
-        <v>2.23</v>
-      </c>
-      <c r="E20">
-        <v>0.02</v>
-      </c>
-      <c r="F20">
-        <v>2.12</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" s="6" customFormat="1">
-      <c r="A21" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="D21" s="6">
-        <v>105</v>
-      </c>
-      <c r="E21" s="6">
+      <c r="B25" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="D25" s="6">
+        <v>22</v>
+      </c>
+      <c r="E25" s="6">
         <v>1</v>
       </c>
-      <c r="F21" s="6">
+      <c r="F25" s="6">
         <v>100</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:F21">
+  <conditionalFormatting sqref="B2:F25">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Imtechella halotolerans">
       <formula>NOT(ISERROR(SEARCH("Imtechella halotolerans",B2)))</formula>
     </cfRule>
@@ -1422,34 +1484,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" s="1" customFormat="1">
-      <c r="A1" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>68</v>
-      </c>
       <c r="H1" s="1" t="s">
         <v>43</v>
       </c>
@@ -1468,80 +1509,80 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2" s="1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="B2" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C2" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="D2" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="E2" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="F2" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="G2" t="s">
-        <v>90</v>
-      </c>
-      <c r="H2">
-        <v>2700</v>
-      </c>
-      <c r="K2">
-        <v>25</v>
+        <v>84</v>
+      </c>
+      <c r="I2">
+        <v>8620</v>
       </c>
     </row>
     <row r="3" spans="1:12">
       <c r="A3" s="1" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B3" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="C3" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="D3" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="E3" t="s">
+        <v>78</v>
+      </c>
+      <c r="F3" t="s">
+        <v>82</v>
+      </c>
+      <c r="G3" t="s">
         <v>84</v>
       </c>
-      <c r="F3" t="s">
-        <v>88</v>
-      </c>
-      <c r="G3" t="s">
-        <v>90</v>
-      </c>
-      <c r="I3">
-        <v>2000</v>
+      <c r="H3">
+        <v>7730</v>
+      </c>
+      <c r="K3">
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:12">
       <c r="A4" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C4" t="s">
         <v>69</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>74</v>
       </c>
-      <c r="D4" t="s">
-        <v>79</v>
-      </c>
       <c r="E4" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="F4" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="G4" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="J4">
         <v>950</v>
@@ -1552,25 +1593,25 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B5" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="C5" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="D5" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="E5" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="F5" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="G5" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="J5">
         <v>50</v>
@@ -1581,104 +1622,75 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B6" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="C6" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="D6" t="s">
+        <v>74</v>
+      </c>
+      <c r="E6" t="s">
+        <v>78</v>
+      </c>
+      <c r="F6" t="s">
         <v>82</v>
       </c>
-      <c r="E6" t="s">
-        <v>86</v>
-      </c>
-      <c r="F6" t="s">
-        <v>86</v>
-      </c>
       <c r="G6" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="L6">
-        <v>50</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:12">
       <c r="A7" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B7" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C7" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="D7" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E7" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F7" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="G7" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="L7">
-        <v>2.77</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8" spans="1:12">
-      <c r="A8" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B8" t="s">
-        <v>73</v>
-      </c>
-      <c r="C8" t="s">
-        <v>78</v>
-      </c>
-      <c r="D8" t="s">
-        <v>79</v>
-      </c>
-      <c r="E8" t="s">
-        <v>83</v>
-      </c>
-      <c r="F8" t="s">
-        <v>87</v>
-      </c>
-      <c r="G8" t="s">
-        <v>90</v>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>1314</v>
       </c>
       <c r="L8">
-        <v>2.23</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12">
-      <c r="A9" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="H9">
-        <v>0</v>
-      </c>
-      <c r="I9">
-        <v>0</v>
-      </c>
-      <c r="J9">
-        <v>0</v>
-      </c>
-      <c r="K9">
-        <v>1500</v>
-      </c>
-      <c r="L9">
-        <v>50</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:F21">
+  <conditionalFormatting sqref="B2:F25">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Imtechella halotolerans">
       <formula>NOT(ISERROR(SEARCH("Imtechella halotolerans",B2)))</formula>
     </cfRule>
@@ -1695,34 +1707,13 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="25.7109375" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" s="1" customFormat="1">
-      <c r="A1" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>68</v>
-      </c>
       <c r="H1" s="1" t="s">
         <v>43</v>
       </c>
@@ -1741,83 +1732,83 @@
     </row>
     <row r="2" spans="1:12">
       <c r="A2" s="1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="B2" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C2" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="D2" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="E2" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="F2" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="G2" t="s">
-        <v>90</v>
-      </c>
-      <c r="H2">
+        <v>84</v>
+      </c>
+      <c r="I2">
         <v>1</v>
-      </c>
-      <c r="K2">
-        <v>0.19</v>
       </c>
     </row>
     <row r="3" spans="1:12">
       <c r="A3" s="1" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B3" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="C3" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="D3" t="s">
-        <v>80</v>
+        <v>74</v>
       </c>
       <c r="E3" t="s">
+        <v>78</v>
+      </c>
+      <c r="F3" t="s">
+        <v>82</v>
+      </c>
+      <c r="G3" t="s">
         <v>84</v>
       </c>
-      <c r="F3" t="s">
-        <v>88</v>
-      </c>
-      <c r="G3" t="s">
-        <v>90</v>
-      </c>
-      <c r="I3">
+      <c r="H3">
         <v>1</v>
+      </c>
+      <c r="K3">
+        <v>0.19</v>
       </c>
     </row>
     <row r="4" spans="1:12">
       <c r="A4" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B4" t="s">
+        <v>64</v>
+      </c>
+      <c r="C4" t="s">
         <v>69</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>74</v>
       </c>
-      <c r="D4" t="s">
-        <v>79</v>
-      </c>
       <c r="E4" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="F4" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="G4" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="J4">
-        <v>0.95</v>
+        <v>95</v>
       </c>
       <c r="K4">
         <v>0.07000000000000001</v>
@@ -1825,28 +1816,28 @@
     </row>
     <row r="5" spans="1:12">
       <c r="A5" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B5" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="C5" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="D5" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="E5" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="F5" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="G5" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="J5">
-        <v>0.05</v>
+        <v>5</v>
       </c>
       <c r="K5">
         <v>0.74</v>
@@ -1854,104 +1845,75 @@
     </row>
     <row r="6" spans="1:12">
       <c r="A6" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B6" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="C6" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="D6" t="s">
+        <v>74</v>
+      </c>
+      <c r="E6" t="s">
+        <v>78</v>
+      </c>
+      <c r="F6" t="s">
         <v>82</v>
       </c>
-      <c r="E6" t="s">
-        <v>86</v>
-      </c>
-      <c r="F6" t="s">
-        <v>86</v>
-      </c>
       <c r="G6" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="L6">
-        <v>0.91</v>
+        <v>0.59</v>
       </c>
     </row>
     <row r="7" spans="1:12">
       <c r="A7" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B7" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C7" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
       <c r="D7" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E7" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="F7" t="s">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="G7" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="L7">
-        <v>0.05</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="8" spans="1:12">
-      <c r="A8" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="B8" t="s">
-        <v>73</v>
-      </c>
-      <c r="C8" t="s">
-        <v>78</v>
-      </c>
-      <c r="D8" t="s">
-        <v>79</v>
-      </c>
-      <c r="E8" t="s">
-        <v>83</v>
-      </c>
-      <c r="F8" t="s">
-        <v>87</v>
-      </c>
-      <c r="G8" t="s">
-        <v>90</v>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
+        <v>0</v>
+      </c>
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
       </c>
       <c r="L8">
-        <v>0.04</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12">
-      <c r="A9" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="H9">
-        <v>0</v>
-      </c>
-      <c r="I9">
-        <v>0</v>
-      </c>
-      <c r="J9">
-        <v>0</v>
-      </c>
-      <c r="K9">
-        <v>0</v>
-      </c>
-      <c r="L9">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:F21">
+  <conditionalFormatting sqref="B2:F25">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Imtechella halotolerans">
       <formula>NOT(ISERROR(SEARCH("Imtechella halotolerans",B2)))</formula>
     </cfRule>

</xml_diff>